<commit_message>
[Fixing] Needing to find accel_file dir twice
เวลาจะเพิ่ม SN จาก PDF เข้ามาใน Accel file มันต้องเพิ่ม Accel มาก่อน แล้ว เพิ่ม pdf หลังจากเพิ่ม pdf ต้องอัพเดทไฟล์โดยการ เพิ่ม Accel File อีกรอบ
</commit_message>
<xml_diff>
--- a/test/jupyter notebook/Accel_mode.xlsx
+++ b/test/jupyter notebook/Accel_mode.xlsx
@@ -1,47 +1,50 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BCP_27\Documents\GitHub\Python\test\jupyter notebook\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0242FC4E-3826-48C2-B772-673D4CEBFEBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="Calc"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="615" yWindow="2760" windowWidth="27030" windowHeight="11295" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <extLst>
+    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
+      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
-    <t>orders</t>
+    <t xml:space="preserve">orders</t>
   </si>
   <si>
-    <t>sn</t>
+    <t xml:space="preserve">sn</t>
   </si>
   <si>
-    <t>240813685HA4NJ</t>
+    <t xml:space="preserve">240813685HA4NJ</t>
   </si>
   <si>
-    <t>2408136AT6NRM5</t>
+    <t xml:space="preserve">2408136AT6NRM5</t>
   </si>
   <si>
-    <t>2408148RNYAJ6T</t>
+    <t xml:space="preserve">2408148RNYAJ6T</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="General"/>
+  </numFmts>
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -50,15 +53,32 @@
       <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="11"/>
       <name val="Cambria"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -71,33 +91,26 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF8F8FF"/>
+        <bgColor rgb="FFF0F0F0"/>
       </patternFill>
     </fill>
   </fills>
   <borders count="3">
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right style="thin">
         <color rgb="FFF0F0F0"/>
@@ -109,73 +122,160 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="20">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+  <cellXfs count="5">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFF8F8FF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFF0F0F0"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1F497D"/>
+        <a:srgbClr val="1f497d"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="EEECE1"/>
+        <a:srgbClr val="eeece1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4F81BD"/>
+        <a:srgbClr val="4f81bd"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="C0504D"/>
+        <a:srgbClr val="c0504d"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9BBB59"/>
+        <a:srgbClr val="9bbb59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064A2"/>
+        <a:srgbClr val="8064a2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4BACC6"/>
+        <a:srgbClr val="4bacc6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="F79646"/>
+        <a:srgbClr val="f79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000FF"/>
+        <a:srgbClr val="0000ff"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -183,12 +283,12 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -217,7 +317,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -238,7 +338,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -289,7 +389,7 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -307,51 +407,56 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="13.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="26.28515625" customWidth="1"/>
-    <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
-    <col min="16296" max="16384" width="11.5703125" customWidth="1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="3.51"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="0" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+    <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+    <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
     </row>
   </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>